<commit_message>
fix:batas atas and akhir first selector
</commit_message>
<xml_diff>
--- a/dataset/pendaftaran_umum.xlsx
+++ b/dataset/pendaftaran_umum.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R21"/>
+  <dimension ref="A1:R33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16" outlineLevelCol="0"/>
   <cols>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -1287,7 +1287,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="17" customHeight="1">
       <c r="A10" s="1" t="inlineStr">
         <is>
           <t>3512075610720001</t>
@@ -1467,7 +1467,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="17" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
           <t>3512076709690002</t>
@@ -1557,7 +1557,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="17" customHeight="1">
       <c r="A13" s="1" t="inlineStr">
         <is>
           <t>3319091108880005</t>
@@ -1647,7 +1647,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="17" customHeight="1">
       <c r="A14" s="1" t="inlineStr">
         <is>
           <t>3512096104830001</t>
@@ -1737,7 +1737,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="17" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
         <is>
           <t>3512060209800002</t>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="17" customHeight="1">
       <c r="A16" s="1" t="inlineStr">
         <is>
           <t>3512134301930006</t>
@@ -1917,7 +1917,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="17" customHeight="1">
       <c r="A17" s="1" t="inlineStr">
         <is>
           <t>3512076508980002</t>
@@ -2007,7 +2007,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="17" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
         <is>
           <t>3505142311880001</t>
@@ -2097,7 +2097,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="17" customHeight="1">
       <c r="A19" s="1" t="inlineStr">
         <is>
           <t>3512074106740002</t>
@@ -2364,6 +2364,1068 @@
       <c r="R21" t="inlineStr">
         <is>
           <t>Jl. Wr Supratman</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>3512072706060001</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>DIYO SAPUTRA</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Pasien ini sudah menerima CKG</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="inlineStr">
+        <is>
+          <t>2006-06-27</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Laki-laki</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="inlineStr">
+        <is>
+          <t>85231961508</t>
+        </is>
+      </c>
+      <c r="G22" s="1" t="inlineStr">
+        <is>
+          <t>3509116303960002</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>sri indriyani</t>
+        </is>
+      </c>
+      <c r="I22" s="1" t="inlineStr">
+        <is>
+          <t>1996-03-23</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Perempuan</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>85231961508</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Menikah</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>ASN (Kantor Pemerintah)</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Jawa Timur</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Kab. Situbondo</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Panarukan</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Sumberkolak</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Sumberkolak</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>3512071107880001</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>IRWAN EFENDI</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Pasien ini sudah menerima CKG</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t>1988-07-11</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Laki-laki</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="n">
+        <v>85231961508</v>
+      </c>
+      <c r="G23" s="1" t="inlineStr">
+        <is>
+          <t>3509116303960002</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>sri indriyani</t>
+        </is>
+      </c>
+      <c r="I23" s="1" t="inlineStr">
+        <is>
+          <t>1996-03-23</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Perempuan</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>85231961508</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Menikah</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>ASN (Kantor Pemerintah)</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Jawa Timur</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Kab. Situbondo</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Situbondo</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Patokan</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Puri Pratama</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>3512074907990007</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>HOLISATUR ROHMAH</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Pasien ini sudah menerima CKG</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="inlineStr">
+        <is>
+          <t>1999-07-09</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Perempuan</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="n">
+        <v>85231961508</v>
+      </c>
+      <c r="G24" s="1" t="inlineStr">
+        <is>
+          <t>3509116303960002</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>sri indriyani</t>
+        </is>
+      </c>
+      <c r="I24" s="1" t="inlineStr">
+        <is>
+          <t>1996-03-23</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Perempuan</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>85231961508</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Menikah</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>ASN (Kantor Pemerintah)</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Jawa Timur</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Kab. Situbondo</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Situbondo</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Patokan</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Jl. Kenanga</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>3512075906690001</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SITI FATIMAH</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Pasien ini sudah menerima CKG</t>
+        </is>
+      </c>
+      <c r="D25" s="1" t="inlineStr">
+        <is>
+          <t>1969-06-19</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Perempuan</t>
+        </is>
+      </c>
+      <c r="F25" s="1" t="n">
+        <v>85231961508</v>
+      </c>
+      <c r="G25" s="1" t="inlineStr">
+        <is>
+          <t>3509116303960002</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>sri indriyani</t>
+        </is>
+      </c>
+      <c r="I25" s="1" t="inlineStr">
+        <is>
+          <t>1996-03-23</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Perempuan</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>85231961508</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Menikah</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>ASN (Kantor Pemerintah)</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Jawa Timur</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Kab. Situbondo</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Situbondo</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Dawuhan</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Dawuhan Parse</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>3512070107780010</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>MISTARI</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Pasien ini sudah menerima CKG</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="inlineStr">
+        <is>
+          <t>1978-07-01</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Laki-laki</t>
+        </is>
+      </c>
+      <c r="F26" s="1" t="n">
+        <v>85231961508</v>
+      </c>
+      <c r="G26" s="1" t="inlineStr">
+        <is>
+          <t>3509116303960002</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>sri indriyani</t>
+        </is>
+      </c>
+      <c r="I26" s="1" t="inlineStr">
+        <is>
+          <t>1996-03-23</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Perempuan</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>85231961508</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Menikah</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>ASN (Kantor Pemerintah)</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Jawa Timur</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Kab. Situbondo</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Situbondo</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Kalibagor</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Kalibagor</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>3512076006850003</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>SUNI YULIANI</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Pasien ini sudah menerima CKG</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="inlineStr">
+        <is>
+          <t>1988-02-01</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Laki-laki</t>
+        </is>
+      </c>
+      <c r="F27" s="1" t="n">
+        <v>85231961508</v>
+      </c>
+      <c r="G27" s="1" t="inlineStr">
+        <is>
+          <t>3509116303960002</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>sri indriyani</t>
+        </is>
+      </c>
+      <c r="I27" s="1" t="inlineStr">
+        <is>
+          <t>1996-03-23</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Perempuan</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>85231961508</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Menikah</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>ASN (Kantor Pemerintah)</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Jawa Timur</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Kab. Situbondo</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Panarukan</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Sumberkolak</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Sumberkolak</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>3512071102790001</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ABU BAKAR</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Pasien ini sudah menerima CKG</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="inlineStr">
+        <is>
+          <t>1979-02-11</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Laki-laki</t>
+        </is>
+      </c>
+      <c r="F28" s="1" t="n">
+        <v>85231961508</v>
+      </c>
+      <c r="G28" s="1" t="inlineStr">
+        <is>
+          <t>3509116303960002</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>sri indriyani</t>
+        </is>
+      </c>
+      <c r="I28" s="1" t="inlineStr">
+        <is>
+          <t>1996-03-23</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Perempuan</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>85231961508</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Menikah</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>ASN (Kantor Pemerintah)</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Jawa Timur</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Kab. Situbondo</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Situbondo</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Kalibagor</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Kalibagor</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>3512075001770008</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>TUMIYATI</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Pasien ini sudah menerima CKG</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="inlineStr">
+        <is>
+          <t>1977-01-10</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Perempuan</t>
+        </is>
+      </c>
+      <c r="F29" s="1" t="n">
+        <v>85231961508</v>
+      </c>
+      <c r="G29" s="1" t="inlineStr">
+        <is>
+          <t>3509116303960002</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>sri indriyani</t>
+        </is>
+      </c>
+      <c r="I29" s="1" t="inlineStr">
+        <is>
+          <t>1996-03-23</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Perempuan</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>85231961508</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Menikah</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>ASN (Kantor Pemerintah)</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Jawa Timur</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Kab. Situbondo</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Situbondo</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Patokan</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Jl. Anggrek</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>3512075702820002</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>SUHAINA</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="inlineStr">
+        <is>
+          <t>1982-02-17</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Perempuan</t>
+        </is>
+      </c>
+      <c r="F30" s="1" t="n">
+        <v>85231961508</v>
+      </c>
+      <c r="G30" s="1" t="inlineStr">
+        <is>
+          <t>3509116303960002</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>sri indriyani</t>
+        </is>
+      </c>
+      <c r="I30" s="1" t="inlineStr">
+        <is>
+          <t>1996-03-23</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Perempuan</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>85231961508</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Menikah</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>ASN (Kantor Pemerintah)</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Jawa Tengah</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Kab. Situbondo</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Situbondo</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Patokan</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Kandang Mas</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>3512075204810005</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>UCIK BING SLAMET</t>
+        </is>
+      </c>
+      <c r="D31" s="1" t="inlineStr">
+        <is>
+          <t>1981-04-01</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Perempuan</t>
+        </is>
+      </c>
+      <c r="F31" s="1" t="n">
+        <v>85231961508</v>
+      </c>
+      <c r="G31" s="1" t="inlineStr">
+        <is>
+          <t>3509116303960002</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>sri indriyani</t>
+        </is>
+      </c>
+      <c r="I31" s="1" t="inlineStr">
+        <is>
+          <t>1996-03-23</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Perempuan</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>85231961508</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Menikah</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>ASN (Kantor Pemerintah)</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Jawa Timur</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Kab. Situbondo</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Situbondo</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Patokan</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Jl. Anggrek</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>3512070107680003</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>MISYADI</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="inlineStr">
+        <is>
+          <t>1968-07-01</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Laki-laki</t>
+        </is>
+      </c>
+      <c r="F32" s="1" t="n">
+        <v>85231961508</v>
+      </c>
+      <c r="G32" s="1" t="inlineStr">
+        <is>
+          <t>3509116303960002</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>sri indriyani</t>
+        </is>
+      </c>
+      <c r="I32" s="1" t="inlineStr">
+        <is>
+          <t>1996-03-23</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Perempuan</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>85231961508</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Menikah</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>ASN (Kantor Pemerintah)</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Jawa Timur</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Kab. Situbondo</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Panarukan</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Perum</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Perum Villa </t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>3512074301840005</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>SUSANTI</t>
+        </is>
+      </c>
+      <c r="D33" s="1" t="inlineStr">
+        <is>
+          <t>1984-01-03</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Perempuan</t>
+        </is>
+      </c>
+      <c r="F33" s="1" t="n">
+        <v>85231961508</v>
+      </c>
+      <c r="G33" s="1" t="inlineStr">
+        <is>
+          <t>3509116303960002</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>sri indriyani</t>
+        </is>
+      </c>
+      <c r="I33" s="1" t="inlineStr">
+        <is>
+          <t>1996-03-23</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Perempuan</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>85231961508</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Menikah</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>ASN (Kantor Pemerintah)</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Jawa Timur</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Kab. Situbondo</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Asembagus</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Asembagus</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Asembagus</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: stage 3/3 of fixing pendaftaran baru fixing complete
</commit_message>
<xml_diff>
--- a/dataset/pendaftaran_umum.xlsx
+++ b/dataset/pendaftaran_umum.xlsx
@@ -848,10 +848,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAILED: Locator.click: Timeout 30000ms exceeded.
-Call log:
-  - waiting for get_by_role("button", name="Tutup")
-</t>
+          <t>SUCCESS</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
@@ -1035,10 +1032,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAILED: Locator.click: Timeout 30000ms exceeded.
-Call log:
-  - waiting for get_by_role("button", name="Tutup")
-</t>
+          <t>SUCCESS</t>
         </is>
       </c>
       <c r="D7" s="1" t="inlineStr">

</xml_diff>

<commit_message>
feat: implement no-click-delay context manager for date picker functionality
</commit_message>
<xml_diff>
--- a/dataset/pendaftaran_umum.xlsx
+++ b/dataset/pendaftaran_umum.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R62"/>
+  <dimension ref="A1:R32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16"/>
   <cols>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -1011,6 +1011,15 @@
       <c r="O18" s="1" t="n"/>
       <c r="Q18" s="1" t="n"/>
     </row>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
     <row r="28" ht="17" customHeight="1">
       <c r="C28" s="2" t="n"/>
     </row>
@@ -1029,666 +1038,6 @@
       <c r="L32" s="1" t="n"/>
       <c r="M32" s="1" t="n"/>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>3512340601117216</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Muhammad Gilang Ardianto</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>2011-01-06</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Laki-laki</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>3512816207098932</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Carla</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>2009-07-22</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Perempuan</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>3512321508103429</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Danu Pradipta</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>2010-08-15</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Laki-laki</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>3512625201111915</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Pia Rahayu Hariyah</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>2011-01-12</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Perempuan</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>3512613101107732</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Jindra Mardhiyah</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>2010-01-31</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Laki-laki</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>3512426506108403</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Diana Kuswandari</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>2010-06-25</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Perempuan</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>3512784101137725</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Hasna Yuni Ramadan</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>2013-01-01</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Perempuan</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>3512235009168538</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Cindy</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>2016-09-10</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Perempuan</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>3512294306166752</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Maida</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>2016-06-03</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Perempuan</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>3512786908099916</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Devi</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>2009-08-29</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Perempuan</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>3512024903105211</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Ayu Kurnia Wibisono</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>2010-03-09</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Perempuan</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>3512534309125834</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Febi Ani Prabowo</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>2012-09-03</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Perempuan</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>3512182504110532</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Nasrullah</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>2011-04-25</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Laki-laki</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>3512751011123761</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Ajimin Melani</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>2012-11-10</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Laki-laki</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>3512961009096522</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Utama Permadi</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>2009-09-10</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Laki-laki</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>3512804205145054</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Zizi Suartini</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>2014-05-02</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Perempuan</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>3512475210138683</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Elma Hutagalung</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>2013-10-12</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Perempuan</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>3512035902122420</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Dian</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>2012-02-19</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Perempuan</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>3512931112105764</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Raditya Ridwan Yuliarti</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>2010-12-11</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Laki-laki</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>3512652411137642</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Gading Lukman Usamah</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>2013-11-24</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Laki-laki</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>3512261111150528</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Liman Irawan</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>2015-11-11</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Laki-laki</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>3512305909107734</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Carla Halimah Santoso</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>2010-09-19</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Perempuan</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>3512520506121671</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Lukita Sihombing</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>2012-06-05</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Laki-laki</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>3512285508159903</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Restu</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>2015-08-15</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Perempuan</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>3512666409168063</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Alika Siska Wijayanti</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>2016-09-24</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Perempuan</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>3512170309150367</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Lamar Nanda Uyainah</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>2015-09-03</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Laki-laki</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>3512994504093839</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Malika Lestari</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>2009-04-05</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Perempuan</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>3512746008151731</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Oni Anggriawan</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>2015-08-20</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Perempuan</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>3512892011165919</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Olga Habibi</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>2016-11-20</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Laki-laki</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>3512732104116505</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Saka</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>2011-04-21</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Laki-laki</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>